<commit_message>
feat(songshan): rebuild data from XLS source + correct device params
Major changes:
- generate_songshan_data.py v3: use project XLS 12m×24h typical day profiles
  instead of temperature-weighted synthesis
- ele_load: non-AC public electricity only (69.59 wan kWh/yr, was 166.64)
- cool_load: demand-side from XLS Table C (291.15 wan kWh/yr)
- cool peak: actual coincident ~2300 kW (clip 3460, was 5797)
- cooling-to-electricity ratio: 4.18 (matches PDF exactly)
- Weekend cooling = 0, electricity same all days (XLS verified)

case_config.py parameter corrections:
- gt_eta_e: 0.35 -> 0.423 (CAT G3512E official spec)
- gt_eta_h: 0.45 -> 0.42 (综合效率80% back-calculation)
- ec_cop: 3.5 -> 5.5 (1500kW chiller industry value)

New files:
- 松山湖/松山湖社区方案-0901.xls (project source data)
- 松山湖/松山湖数据保存/10_XLS源数据提取.md
- 松山湖/松山湖数据保存/11_XLS数据讲解.md
</commit_message>
<xml_diff>
--- a/data/songshan_lake_typical.xlsx
+++ b/data/songshan_lake_typical.xlsx
@@ -447,183 +447,183 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>106</v>
+        <v>252</v>
       </c>
       <c r="B2" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>91,92,93,94,95,96,97,98,99,100,101,102,103,104,105,106,107,108,109,110,111,112,113,114,115,116,117,118,119,120</t>
+          <t>194,208,213,216,217,221,228,230,238,242,243,244,245,248,249,250,252,256,257,258,264,265,266,269,270,271,272,273</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="B3" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>121,122,123,124,125,126,127,128,129,130,131,132,133,134,135,136,137,138,139,140,141,142,143,144,145,146,147,148,149,150,151</t>
+          <t>124,129,144,145,147,151,152,157,158,159,160,164,165,166,168,172,178,179,180,181</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>257</v>
+        <v>241</v>
       </c>
       <c r="B4" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>244,245,246,247,248,249,250,251,252,253,254,255,256,257,258,259,260,261,262,263,264,265,266,267,268,269,270,271,272,273</t>
+          <t>153,154,161,167,171,173,174,175,182,185,186,187,188,189,192,193,195,196,199,200,201,202,203,206,207,209,210,214,215,220,222,223,224,227,229,231,234,235,236,237,241,251,255,259,262,263</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>222</v>
+        <v>133</v>
       </c>
       <c r="B5" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>186,213,214,215,218,219,220,221,222,223,225,226,227,228,229,233,234,235,236,239,240,241,242,243</t>
+          <t>122,123,125,126,130,131,132,133,136,137,138,139,140,143,146,150</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>155</v>
+        <v>103</v>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>152,153,155,156,157,159,160,162,163,164,166,167,168,169,170,172,173,174,176,178,180,181</t>
+          <t>91,92,93,94,95,96,97,98,99,100,101,102,103,104,105,106,107,108,109,110,111,112,113,114,115,116,117,118,119,120</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>217</v>
+        <v>240</v>
       </c>
       <c r="B7" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>154,158,161,165,171,175,177,179,182,183,184,185,187,188,189,190,191,192,193,194,195,196,197,198,199,200,201,202,203,204,205,206,207,208,209,210,211,212,216,217,224,230,231,232,237,238</t>
+          <t>127,148,204,211,212,240,253,260,268</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>17</v>
+        <v>155</v>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
+          <t>121,128,134,135,141,142,149,155,156,162,163,169,170,176,177,183,184,190,191,197,198,205,218,219,225,226,232,233,239,246,247,254,261,267</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>68</v>
+        <v>326</v>
       </c>
       <c r="B9" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>60,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,87,88,89,90</t>
+          <t>306,307,311,312,313,314,318,319,320,321,322,325,326,328,329,332,333</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="B10" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>32,33,34,35,36,37,38,39,40,41,42,43,44,45,46,47,48,49,50,51,52,53,54,55,56,57,58,59</t>
+          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>339</v>
+        <v>41</v>
       </c>
       <c r="B11" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>337,338,339,340,341,345,346,347,351,352,353,354,355,358,359,360,361,362,365</t>
+          <t>32,36,37,39,40,41,45,46,50,51,55,56,57,310,324,330,331</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>350</v>
+        <v>74</v>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>335,336,342,343,344,348,349,350,356,357,363,364</t>
+          <t>33,34,35,38,42,43,44,47,48,49,52,53,54,58,59,60,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,87,88,89,90,305,308,309,315,316,317,323,327,334</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>291</v>
+        <v>364</v>
       </c>
       <c r="B13" t="n">
         <v>31</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>274,275,276,277,278,279,280,281,282,283,284,285,286,287,288,289,290,291,292,293,294,295,296,297,298,299,300,301,302,303,304</t>
+          <t>335,336,337,338,339,340,341,342,343,344,345,346,347,348,349,350,351,352,353,354,355,356,357,358,359,360,361,362,363,364,365</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>319</v>
+        <v>289</v>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>316,318,319,324,328,333</t>
+          <t>274,275,281,282,288,289,295,296,302,303</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>320</v>
+        <v>290</v>
       </c>
       <c r="B15" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>305,306,307,308,309,310,311,312,313,314,315,317,320,321,322,323,325,326,327,329,330,331,332,334</t>
+          <t>276,277,278,279,280,283,284,285,286,287,290,291,292,293,294,297,298,299,300,301,304</t>
         </is>
       </c>
     </row>

</xml_diff>